<commit_message>
Cierra ingeniería y análisis del dato del TFG
</commit_message>
<xml_diff>
--- a/analisis_dato/data/analytic/summary/master_results_table.xlsx
+++ b/analisis_dato/data/analytic/summary/master_results_table.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,47 +424,72 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>subcapa</t>
+          <t>bloque</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>tipo_modelo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>objetivo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>modelo</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>muestra</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>metricas_clave</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>resultado_principal</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>interpretacion_breve</t>
+          <t>mae</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>test_f1</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>test_auc</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>gap_f1</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>interpretacion</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>estado</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>es_ganador</t>
         </is>
       </c>
     </row>
@@ -476,100 +501,118 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Macro temporal retail moda</t>
+          <t>Series temporales — Retail moda</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Predecir la evolución del índice retail moda</t>
+          <t>regresion_temporal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Predecir evolución del índice retail moda (base 2015=100)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>capa1_master_mensual_analysis.csv</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>SARIMA(0,1,1)(0,1,0,12)</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Principal</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>MAE=5.978 | RMSE=8.953 | MAPE=4.750</t>
+          <t>Avanzado (Ganador)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Modelo temporal final seleccionado tras tuning</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Capta la evolución temporal del retail moda y sirve como marco macro del consumo.</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
+          <t>MAE=5.978 | RMSE=8.953 | MAPE=4.75%</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>5.978047182420763</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Serie temporal con estacionalidad mensual. Captura patrón rebajas y navidad.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>Final</t>
         </is>
+      </c>
+      <c r="O2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Capa 2</t>
+          <t>Capa 1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2A - Instagram engagement</t>
+          <t>Series temporales — Retail moda</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Predecir publicaciones con alto engagement</t>
+          <t>regresion_temporal</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>instagram_model_input.csv</t>
+          <t>Predecir evolución del índice retail moda (base 2015=100)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>capa1_master_mensual_analysis.csv</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Holt-Winters_ETS-AAA</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Accuracy=0.882 | F1=0.761 | ROC_AUC=0.907</t>
+          <t>Baseline</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Comparación de modelos supervisados para engagement alto</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Permite identificar patrones de publicación asociados a mayor respuesta del público.</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
+          <t>MAE=17.882 | RMSE=21.410 | MAPE=14.40%</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>17.88225001463948</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Serie temporal con estacionalidad mensual. Captura patrón rebajas y navidad.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>Final</t>
         </is>
+      </c>
+      <c r="O3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -580,48 +623,61 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2A - Instagram engagement</t>
+          <t>2A — Clasificación engagement Instagram</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Predecir publicaciones con alto engagement</t>
+          <t>clasificacion_supervisada</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>Predecir publicaciones con alto engagement (&gt; P75)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>instagram_model_input.csv</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>logistic_regression</t>
-        </is>
-      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>B_Random_Forest</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Accuracy=0.876 | F1=0.738 | ROC_AUC=0.856</t>
+          <t>Avanzado (Ganador)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Comparación de modelos supervisados para engagement alto</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Permite identificar patrones de publicación asociados a mayor respuesta del público.</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
+          <t>Acc=0.882 | F1=0.761 | AUC=0.905 | Gap_F1=-0.011</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="n">
+        <v>0.7606837606837606</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.9050418967815655</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-0.0114774114774114</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Predice alto engagement a partir de marca, tipo de post y estacionalidad.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>Final</t>
         </is>
+      </c>
+      <c r="O4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -632,48 +688,61 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2A - Instagram engagement</t>
+          <t>2A — Clasificación engagement Instagram</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Refinar la predicción de publicaciones con alto engagement</t>
+          <t>clasificacion_supervisada</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>Predecir publicaciones con alto engagement (&gt; P75)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>instagram_model_input.csv</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>random_forest_v2</t>
-        </is>
-      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Iteración adicional</t>
+          <t>A_Logistic_Regression</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Accuracy=0.882 | F1=0.761 | ROC_AUC=0.905</t>
+          <t>Baseline</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Segunda iteración de comparación</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Sirve para contrastar estabilidad del rendimiento y robustez del enfoque.</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Complementario</t>
-        </is>
+          <t>Acc=0.876 | F1=0.738 | AUC=0.862 | Gap_F1=-0.020</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="n">
+        <v>0.7377777777777778</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.8622167206246429</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-0.0195457335788826</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Predice alto engagement a partir de marca, tipo de post y estacionalidad.</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="O5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -684,48 +753,61 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2A - Instagram engagement</t>
+          <t>2B — Text Mining captions Instagram</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Refinar la predicción de publicaciones con alto engagement</t>
+          <t>text_mining_clasificacion</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>instagram_model_input.csv</t>
+          <t>Predecir alto engagement a partir del texto del caption (TF-IDF)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>logistic_regression_v2</t>
+          <t>instagram_posts_clean.csv (captions)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Iteración adicional</t>
+          <t>A_TFIDF_LogisticRegression</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Accuracy=0.876 | F1=0.738 | ROC_AUC=0.862</t>
+          <t>Baseline (Ganador)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Segunda iteración de comparación</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Sirve para contrastar estabilidad del rendimiento y robustez del enfoque.</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Complementario</t>
-        </is>
+          <t>Acc=0.822 | F1=0.656 | AUC=0.852</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="n">
+        <v>0.6557377049180327</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.8523052846996509</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.0748374716712709</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>TF-IDF + modelo. Identifica términos predictivos del engagement.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="O6" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -736,100 +818,122 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2B - Google Trends Zara</t>
+          <t>2B — Text Mining captions Instagram</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Predecir la evolución temporal del interés de búsqueda de Zara</t>
+          <t>text_mining_clasificacion</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>trends_marcas_clean.csv</t>
+          <t>Predecir alto engagement a partir del texto del caption (TF-IDF)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ARIMA(2,1,2)</t>
+          <t>instagram_posts_clean.csv (captions)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>B_TFIDF_RandomForest</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MAE=4.778 | RMSE=5.382 | MAPE=8.915</t>
+          <t>Avanzado</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Modelo ARIMA final para Zara</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Aproxima la persistencia del interés digital por una marca líder de moda.</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
+          <t>Acc=0.731 | F1=0.575 | AUC=0.834</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>0.5752508361204013</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.8343324906705188</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.0993254350660394</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>TF-IDF + modelo. Identifica términos predictivos del engagement.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
         <is>
           <t>Final</t>
         </is>
+      </c>
+      <c r="O7" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Capa 3</t>
+          <t>Capa 2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Supervisado consumidor</t>
+          <t>2C — Series temporales Google Trends Zara</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Predecir si el consumidor seguirá comprando</t>
+          <t>regresion_temporal</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>capa3_supervised_ready.csv</t>
+          <t>Predecir interés de búsqueda de Zara (Google Trends)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>logistic_regression_main</t>
+          <t>trends_marcas_clean.csv</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>ARIMA(2,1,2)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Test_F1=0.766 | Test_AUC=0.943 | Gap_F1=0.065</t>
+          <t>Final (Ganador)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Evaluación principal sobre muestra observada</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Contrasta capacidad predictiva y estabilidad de modelos sobre comportamiento futuro declarado.</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
+          <t>MAE=4.778 | RMSE=5.382 | MAPE=8.92%</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>4.778133890581144</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>ARIMA seleccionado por menor RMSE en test (2025). Captura tendencia del interés digital.</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>Final</t>
         </is>
+      </c>
+      <c r="O8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -840,48 +944,55 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Supervisado consumidor</t>
+          <t>3A — Clustering consumidores</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Predecir si el consumidor seguirá comprando</t>
+          <t>clustering_no_supervisado</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>capa3_supervised_ready.csv</t>
+          <t>Identificar perfiles naturales de consumidor de moda en RRSS</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>random_forest_main</t>
+          <t>capa3_clustering_ready.csv</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>KMeans k=2</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Test_F1=0.744 | Test_AUC=0.920 | Gap_F1=0.118</t>
+          <t>No supervisado (Ganador)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Evaluación principal sobre muestra observada</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Contrasta capacidad predictiva y estabilidad de modelos sobre comportamiento futuro declarado.</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
+          <t>Silhouette=0.353 | Inercia=1333.0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>El análisis K-Means identifica 2 perfiles diferenciados de consumidor construidos exclusivamente a partir de 7 índices compuestos que sintetizan la influencia de las RRSS, el impulso de compra, la confianza en influencers, la difusión del fast fashion, la experiencia postcompra y el riesgo de arrepentimiento. El Silhouette Score de 0.353 indica una separación buena entre clústeres. Las variables demográficas y de conducta se reservan para la caracterización posterior de los segmentos, evitando que dominen artificialmente la segmentación.</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
         <is>
           <t>Final</t>
         </is>
+      </c>
+      <c r="O9" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -892,48 +1003,61 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Supervisado consumidor</t>
+          <t>3B — Clasificación intención de compra futura</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Comprobar robustez del modelo al equilibrar generaciones</t>
+          <t>clasificacion_supervisada</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>capa3_supervised_balanced_generation.csv</t>
+          <t>Predecir si el consumidor seguirá comprando influido por RRSS</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>random_forest_balanced</t>
+          <t>capa3_supervised_ready.csv</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Balanceada por generación</t>
+          <t>A_Logistic_Regression</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Test_F1=0.690 | Test_AUC=0.893 | Gap_F1=0.137</t>
+          <t>Baseline (Ganador)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Análisis de sensibilidad por estructura generacional</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Permite comprobar cuánto dependen los resultados del peso de Gen Z en la muestra.</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Robustez</t>
-        </is>
+          <t>Acc=0.828 | F1=0.766 | AUC=0.943 | Gap_F1=0.065</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>0.7659574468085106</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.942690058479532</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.0653678543963086</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Predice intención de compra futura a partir de índices psicológicos e índices de influencia RRSS.</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="O10" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -944,204 +1068,61 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Supervisado consumidor</t>
+          <t>3B — Clasificación intención de compra futura</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Comprobar robustez del modelo al equilibrar generaciones</t>
+          <t>clasificacion_supervisada</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>capa3_supervised_balanced_generation.csv</t>
+          <t>Predecir si el consumidor seguirá comprando influido por RRSS</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>logistic_regression_balanced</t>
+          <t>capa3_supervised_ready.csv</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Balanceada por generación</t>
+          <t>B_Random_Forest</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Test_F1=0.741 | Test_AUC=0.870 | Gap_F1=0.059</t>
+          <t>Avanzado</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Análisis de sensibilidad por estructura generacional</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Permite comprobar cuánto dependen los resultados del peso de Gen Z en la muestra.</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Robustez</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Capa 3</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Clustering consumidor</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Identificar perfiles de consumidor</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>capa3_clustering_ready.csv</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>KMeans</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Principal</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>k=2 | Silhouette=0.252 | Inercia=3337.813</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Solución final de 2 clústeres</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Distingue entre consumidor digital influenciado y perfil más moderado de baja influencia digital.</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
+          <t>Acc=0.844 | F1=0.773 | AUC=0.927 | Gap_F1=0.046</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="n">
+        <v>0.7727272727272727</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.9274853801169592</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.0459861775651249</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Predice intención de compra futura a partir de índices psicológicos e índices de influencia RRSS.</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>Final</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Capa 3</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Clustering consumidor</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Comprobar robustez de la segmentación al equilibrar generaciones</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>capa3_clustering_balanced_generation.csv</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>KMeans</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Balanceada por generación</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>k=2 | Silhouette=0.256 | Inercia=2247.968</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>La solución k=2 se mantiene al equilibrar la muestra</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Refuerza la solidez de la segmentación y reduce el riesgo de sesgo por sobrerrepresentación generacional.</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Robustez</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Capa 3</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Clustering consumidor</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Explorar una subdivisión adicional de perfiles</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>capa3_clustering_ready.csv</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>KMeans k=3</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Exploratorio</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Análisis visual en PCA 2D + tamaños de clúster</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Sugiere perfiles bajo, intermedio y alto de influencia digital</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Útil como exploración, aunque se mantiene k=2 como solución final por parsimonia y respaldo cuantitativo.</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Exploratorio</t>
-        </is>
+      <c r="O11" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>